<commit_message>
Enable image generation model tests
</commit_message>
<xml_diff>
--- a/ModelEvalApp/Defaults/AI_model_variants.xlsx
+++ b/ModelEvalApp/Defaults/AI_model_variants.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet 1 - AI_model_variants" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1 - AI_model_variants" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -1276,7 +1276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AY22"/>
+  <dimension ref="A1:BD23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.33333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="13.6719" customWidth="1" style="1" min="1" max="1"/>
@@ -1594,6 +1594,31 @@
           <t>translation_speed_score</t>
         </is>
       </c>
+      <c r="AZ2" s="3" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="BA2" s="3" t="inlineStr">
+        <is>
+          <t>Provider Type</t>
+        </is>
+      </c>
+      <c r="BB2" s="3" t="inlineStr">
+        <is>
+          <t>Capabilities</t>
+        </is>
+      </c>
+      <c r="BC2" s="3" t="inlineStr">
+        <is>
+          <t>API Key Env</t>
+        </is>
+      </c>
+      <c r="BD2" s="3" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20.25" customHeight="1" s="14">
       <c r="A3" s="4" t="inlineStr">
@@ -4753,6 +4778,128 @@
       </c>
       <c r="AY22" s="13" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>GPT Image 2</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>gpt-image-2</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n"/>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>OpenAI Image API model; requires OPENAI_API_KEY and image-model account access.</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>per image</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>image generation and image edits</t>
+        </is>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M23" s="13" t="n"/>
+      <c r="N23" s="13" t="n"/>
+      <c r="O23" s="13" t="n"/>
+      <c r="P23" s="13" t="n"/>
+      <c r="Q23" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="R23" s="13" t="n"/>
+      <c r="S23" s="13" t="n"/>
+      <c r="T23" s="13" t="n"/>
+      <c r="U23" s="13" t="n"/>
+      <c r="V23" s="13" t="n"/>
+      <c r="W23" s="13" t="n"/>
+      <c r="X23" s="13" t="n"/>
+      <c r="Y23" s="13" t="n"/>
+      <c r="Z23" s="13" t="n"/>
+      <c r="AA23" s="13" t="n"/>
+      <c r="AB23" s="13" t="n"/>
+      <c r="AC23" s="13" t="n"/>
+      <c r="AD23" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AE23" s="13" t="n"/>
+      <c r="AF23" s="13" t="n"/>
+      <c r="AG23" s="13" t="n"/>
+      <c r="AH23" s="13" t="n"/>
+      <c r="AI23" s="13" t="n"/>
+      <c r="AJ23" s="13" t="n"/>
+      <c r="AK23" s="13" t="n"/>
+      <c r="AL23" s="13" t="n"/>
+      <c r="AM23" s="13" t="n"/>
+      <c r="AN23" s="13" t="n"/>
+      <c r="AO23" s="13" t="n"/>
+      <c r="AP23" s="13" t="n"/>
+      <c r="AQ23" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="AR23" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="AS23" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="AT23" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="AU23" s="13" t="n"/>
+      <c r="AV23" s="13" t="n"/>
+      <c r="AW23" s="13" t="n"/>
+      <c r="AX23" s="13" t="n"/>
+      <c r="AY23" s="13" t="n"/>
+      <c r="AZ23" t="inlineStr">
+        <is>
+          <t>openai_images</t>
+        </is>
+      </c>
+      <c r="BA23" t="inlineStr">
+        <is>
+          <t>openai_image_generation</t>
+        </is>
+      </c>
+      <c r="BB23" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="BC23" t="inlineStr">
+        <is>
+          <t>OPENAI_API_KEY</t>
+        </is>
+      </c>
+      <c r="BD23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>